<commit_message>
update spot_counts metadata files for figs 1-3
</commit_message>
<xml_diff>
--- a/01_nocodazole_treatments/raw_spot_counts_analysis/TableS4_nocodazole_treatment.xlsx
+++ b/01_nocodazole_treatments/raw_spot_counts_analysis/TableS4_nocodazole_treatment.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nalytorres/Documents/GitHub/ERM1_TorresMangual/01_nocodazole_treatments/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nalytorres/Documents/GitHub/ERM1_TorresMangual/01_nocodazole_treatments/raw_spot_counts_analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17EB1B87-EE9A-7047-863F-0B87D446EC7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92CEB690-FD78-B442-8A73-129CBF45A1D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="22020" windowHeight="17660" xr2:uid="{2E47865C-5B6A-2C4D-BA8F-0F652FA7F24F}"/>
+    <workbookView xWindow="5940" yWindow="680" windowWidth="22340" windowHeight="17660" xr2:uid="{2E47865C-5B6A-2C4D-BA8F-0F652FA7F24F}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="4" r:id="rId1"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="111">
   <si>
     <t>mean</t>
   </si>
@@ -349,13 +349,113 @@
   </si>
   <si>
     <t>set-3 mRNA</t>
+  </si>
+  <si>
+    <t>unique identifier of image: date_misc_strain_treatment_imageNumber</t>
+  </si>
+  <si>
+    <t>longer image ID. Redundant with above</t>
+  </si>
+  <si>
+    <t>treatment condition</t>
+  </si>
+  <si>
+    <t>total number of spots per embryo - as reported with WormLib</t>
+  </si>
+  <si>
+    <t>mean total number of mRNA molecules per embryo averaged across all embryos</t>
+  </si>
+  <si>
+    <t>standard deviation of the mean above</t>
+  </si>
+  <si>
+    <t>number of embryos per condition, across 3 reps</t>
+  </si>
+  <si>
+    <t>mRNA species observed by smFISH</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>standard error of the mean —</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> estimate of how much your sample mean would vary if you repeated the experiment with new samples from the same population</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>The mRNA species being tested (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>erm-1 mRNA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> or </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>set-3 mRNA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> — total molecule counts).</t>
+    </r>
+  </si>
+  <si>
+    <t>The Wilcoxon rank sum (W) test statistic, based on the sum of ranks between the two groups.</t>
+  </si>
+  <si>
+    <t>Specifies a two-sided test — checking for a difference between groups in either direction, without assuming which group would be higher.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Probability of observing a difference this extreme if there were truly no difference between groups. </t>
+  </si>
+  <si>
+    <t>Wilcoxon rank sum test with continuity correction, a non-parametric comparison of two independent groups; the continuity correction adjusts the p-value approximation when ties are present or sample sizes are small.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="16">
+  <fonts count="19">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -468,6 +568,24 @@
       <name val="Lucida Sans"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Lucida Sans"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -489,7 +607,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -507,31 +625,34 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -935,30 +1056,30 @@
       <c r="A10" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="B10" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="13"/>
+      <c r="C10" s="22"/>
       <c r="D10" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="7"/>
-      <c r="B11" s="14" t="s">
+      <c r="B11" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="C11" s="14"/>
+      <c r="C11" s="27"/>
       <c r="D11" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="6"/>
-      <c r="B12" s="13" t="s">
+      <c r="B12" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="13"/>
+      <c r="C12" s="22"/>
       <c r="D12" t="s">
         <v>17</v>
       </c>
@@ -981,10 +1102,10 @@
       <c r="C15" s="2"/>
     </row>
     <row r="16" spans="1:4">
-      <c r="A16" s="13" t="s">
+      <c r="A16" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="B16" s="13"/>
+      <c r="B16" s="22"/>
       <c r="C16" s="9" t="s">
         <v>10</v>
       </c>
@@ -993,100 +1114,114 @@
       </c>
     </row>
     <row r="17" spans="1:16">
-      <c r="A17" s="15" t="s">
+      <c r="A17" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="B17" s="15"/>
+      <c r="B17" s="24"/>
       <c r="C17" s="2" t="s">
         <v>89</v>
       </c>
+      <c r="D17" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="18" spans="1:16">
-      <c r="A18" s="15" t="s">
+      <c r="A18" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="B18" s="15"/>
-      <c r="C18" s="21" t="s">
+      <c r="B18" s="24"/>
+      <c r="C18" s="16" t="s">
         <v>81</v>
       </c>
-      <c r="D18" s="2"/>
-      <c r="H18" s="20"/>
-      <c r="I18" s="20"/>
-      <c r="J18" s="20"/>
-      <c r="K18" s="20"/>
-      <c r="L18" s="20"/>
+      <c r="D18" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="H18" s="15"/>
+      <c r="I18" s="15"/>
+      <c r="J18" s="15"/>
+      <c r="K18" s="15"/>
+      <c r="L18" s="15"/>
     </row>
     <row r="19" spans="1:16">
-      <c r="A19" s="15" t="s">
+      <c r="A19" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="15"/>
-      <c r="C19" s="21" t="s">
+      <c r="B19" s="24"/>
+      <c r="C19" s="16" t="s">
         <v>81</v>
       </c>
-      <c r="H19" s="21"/>
-      <c r="I19" s="21"/>
-      <c r="J19" s="21"/>
-      <c r="K19" s="21"/>
-      <c r="L19" s="21"/>
-      <c r="M19" s="20"/>
-      <c r="N19" s="20"/>
-      <c r="O19" s="23"/>
-      <c r="P19" s="23"/>
+      <c r="D19" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="H19" s="16"/>
+      <c r="I19" s="16"/>
+      <c r="J19" s="16"/>
+      <c r="K19" s="16"/>
+      <c r="L19" s="16"/>
+      <c r="M19" s="15"/>
+      <c r="N19" s="15"/>
+      <c r="O19" s="20"/>
+      <c r="P19" s="20"/>
     </row>
     <row r="20" spans="1:16">
-      <c r="A20" s="15" t="s">
+      <c r="A20" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="B20" s="15"/>
+      <c r="B20" s="24"/>
       <c r="C20" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="L20" s="21"/>
-      <c r="M20" s="21"/>
-      <c r="N20" s="21"/>
-      <c r="O20" s="23"/>
-      <c r="P20" s="23"/>
+      <c r="D20" t="s">
+        <v>98</v>
+      </c>
+      <c r="L20" s="16"/>
+      <c r="M20" s="16"/>
+      <c r="N20" s="16"/>
+      <c r="O20" s="20"/>
+      <c r="P20" s="20"/>
     </row>
     <row r="21" spans="1:16">
-      <c r="A21" s="15" t="s">
+      <c r="A21" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="B21" s="15"/>
+      <c r="B21" s="24"/>
       <c r="C21" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="L21" s="22"/>
-      <c r="M21" s="22"/>
-      <c r="N21" s="22"/>
-      <c r="O21" s="22"/>
-      <c r="P21" s="22"/>
+      <c r="D21" t="s">
+        <v>99</v>
+      </c>
+      <c r="L21" s="17"/>
+      <c r="M21" s="17"/>
+      <c r="N21" s="17"/>
+      <c r="O21" s="17"/>
+      <c r="P21" s="17"/>
     </row>
     <row r="22" spans="1:16">
-      <c r="A22" s="15"/>
-      <c r="B22" s="15"/>
+      <c r="A22" s="24"/>
+      <c r="B22" s="24"/>
       <c r="C22" s="2"/>
-      <c r="L22" s="22"/>
-      <c r="M22" s="22"/>
-      <c r="N22" s="22"/>
-      <c r="O22" s="22"/>
-      <c r="P22" s="22"/>
+      <c r="L22" s="17"/>
+      <c r="M22" s="17"/>
+      <c r="N22" s="17"/>
+      <c r="O22" s="17"/>
+      <c r="P22" s="17"/>
     </row>
     <row r="23" spans="1:16">
-      <c r="L23" s="22"/>
-      <c r="M23" s="22"/>
-      <c r="N23" s="22"/>
-      <c r="O23" s="22"/>
-      <c r="P23" s="22"/>
+      <c r="L23" s="17"/>
+      <c r="M23" s="17"/>
+      <c r="N23" s="17"/>
+      <c r="O23" s="17"/>
+      <c r="P23" s="17"/>
     </row>
     <row r="24" spans="1:16" ht="20">
-      <c r="A24" s="17" t="s">
+      <c r="A24" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="B24" s="17"/>
-      <c r="L24" s="22"/>
-      <c r="M24" s="22"/>
-      <c r="N24" s="22"/>
+      <c r="B24" s="26"/>
+      <c r="L24" s="17"/>
+      <c r="M24" s="17"/>
+      <c r="N24" s="17"/>
     </row>
     <row r="25" spans="1:16">
       <c r="A25" s="25" t="s">
@@ -1101,171 +1236,198 @@
       </c>
     </row>
     <row r="26" spans="1:16">
-      <c r="A26" s="20" t="s">
+      <c r="A26" s="15" t="s">
         <v>77</v>
       </c>
-      <c r="C26" s="21" t="s">
+      <c r="C26" s="16" t="s">
         <v>78</v>
       </c>
-      <c r="D26" s="20"/>
-      <c r="E26" s="20"/>
-      <c r="F26" s="20"/>
+      <c r="D26" s="18" t="s">
+        <v>104</v>
+      </c>
+      <c r="E26" s="15"/>
+      <c r="F26" s="15"/>
     </row>
     <row r="27" spans="1:16">
-      <c r="A27" s="20" t="s">
+      <c r="A27" s="15" t="s">
         <v>79</v>
       </c>
-      <c r="C27" s="21" t="s">
+      <c r="C27" s="16" t="s">
         <v>78</v>
       </c>
-      <c r="D27" s="21"/>
-      <c r="E27" s="21"/>
-      <c r="F27" s="21"/>
+      <c r="D27" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="E27" s="16"/>
+      <c r="F27" s="16"/>
     </row>
     <row r="28" spans="1:16">
-      <c r="A28" s="20" t="s">
+      <c r="A28" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="C28" s="21" t="s">
+      <c r="C28" s="16" t="s">
         <v>86</v>
       </c>
-      <c r="D28" s="21"/>
-      <c r="E28" s="21"/>
-      <c r="F28" s="21"/>
+      <c r="D28" t="s">
+        <v>101</v>
+      </c>
     </row>
     <row r="29" spans="1:16">
-      <c r="A29" s="20" t="s">
+      <c r="A29" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="C29" s="21" t="s">
+      <c r="C29" s="16" t="s">
         <v>86</v>
       </c>
-      <c r="D29" s="21"/>
-      <c r="E29" s="21"/>
-      <c r="F29" s="21"/>
+      <c r="D29" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="30" spans="1:16">
-      <c r="A30" s="20" t="s">
+      <c r="A30" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="C30" s="21" t="s">
+      <c r="C30" s="16" t="s">
         <v>81</v>
       </c>
-      <c r="D30" s="21"/>
-      <c r="E30" s="21"/>
-      <c r="F30" s="21"/>
+      <c r="D30" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="E30" s="16"/>
+      <c r="F30" s="16"/>
     </row>
     <row r="31" spans="1:16">
-      <c r="A31" s="20" t="s">
+      <c r="A31" s="15" t="s">
         <v>87</v>
       </c>
-      <c r="C31" s="21" t="s">
+      <c r="C31" s="16" t="s">
         <v>86</v>
       </c>
-      <c r="D31" s="21"/>
-      <c r="E31" s="21"/>
-      <c r="F31" s="21"/>
+      <c r="D31" s="19" t="s">
+        <v>105</v>
+      </c>
+      <c r="E31" s="16"/>
+      <c r="F31" s="16"/>
     </row>
     <row r="32" spans="1:16">
-      <c r="A32" s="20"/>
-      <c r="B32" s="21"/>
-      <c r="C32" s="21"/>
-      <c r="D32" s="21"/>
-      <c r="E32" s="21"/>
-      <c r="F32" s="21"/>
+      <c r="A32" s="15"/>
+      <c r="B32" s="16"/>
+      <c r="C32" s="16"/>
+      <c r="D32" s="16"/>
+      <c r="E32" s="16"/>
+      <c r="F32" s="16"/>
     </row>
     <row r="33" spans="1:13">
-      <c r="A33" s="15"/>
-      <c r="B33" s="15"/>
+      <c r="A33" s="24"/>
+      <c r="B33" s="24"/>
     </row>
     <row r="35" spans="1:13" ht="20">
-      <c r="A35" s="16" t="s">
+      <c r="A35" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="B35" s="16"/>
+      <c r="B35" s="23"/>
     </row>
     <row r="36" spans="1:13">
-      <c r="A36" s="13" t="s">
+      <c r="A36" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B36" s="13"/>
-      <c r="C36" s="9" t="s">
+      <c r="B36" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="D36" s="12" t="s">
+      <c r="C36" s="7" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="37" spans="1:13">
-      <c r="A37" s="20" t="s">
+    <row r="37" spans="1:13" ht="17">
+      <c r="A37" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="B37" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="C37" t="s">
+        <v>106</v>
+      </c>
+      <c r="I37" s="21"/>
+      <c r="J37" s="15"/>
+      <c r="K37" s="15"/>
+      <c r="L37" s="15"/>
+      <c r="M37" s="15"/>
+    </row>
+    <row r="38" spans="1:13" ht="17">
+      <c r="A38" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="C37" s="21" t="s">
+      <c r="B38" s="16" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="38" spans="1:13">
-      <c r="A38" s="20" t="s">
+      <c r="C38" t="s">
+        <v>107</v>
+      </c>
+      <c r="I38" s="21"/>
+      <c r="J38" s="16"/>
+      <c r="K38" s="16"/>
+      <c r="L38" s="16"/>
+      <c r="M38" s="16"/>
+    </row>
+    <row r="39" spans="1:13" ht="17">
+      <c r="A39" s="28" t="s">
         <v>90</v>
       </c>
-      <c r="C38" s="21" t="s">
+      <c r="B39" s="16" t="s">
         <v>86</v>
       </c>
-      <c r="I38" s="24"/>
-      <c r="J38" s="20"/>
-      <c r="K38" s="20"/>
-      <c r="L38" s="20"/>
-      <c r="M38" s="20"/>
-    </row>
-    <row r="39" spans="1:13">
-      <c r="A39" s="20" t="s">
+      <c r="C39" t="s">
+        <v>109</v>
+      </c>
+      <c r="I39" s="17"/>
+      <c r="J39" s="17"/>
+      <c r="K39" s="17"/>
+      <c r="L39" s="17"/>
+      <c r="M39" s="17"/>
+    </row>
+    <row r="40" spans="1:13" ht="17">
+      <c r="A40" s="28" t="s">
         <v>91</v>
       </c>
-      <c r="C39" s="21" t="s">
+      <c r="B40" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="I39" s="24"/>
-      <c r="J39" s="21"/>
-      <c r="K39" s="21"/>
-      <c r="L39" s="21"/>
-      <c r="M39" s="21"/>
-    </row>
-    <row r="40" spans="1:13">
-      <c r="A40" s="20" t="s">
+      <c r="C40" t="s">
+        <v>110</v>
+      </c>
+      <c r="I40" s="17"/>
+      <c r="J40" s="17"/>
+      <c r="K40" s="17"/>
+      <c r="L40" s="17"/>
+      <c r="M40" s="17"/>
+    </row>
+    <row r="41" spans="1:13" ht="17">
+      <c r="A41" s="28" t="s">
         <v>92</v>
       </c>
-      <c r="C40" s="21" t="s">
+      <c r="B41" t="s">
         <v>89</v>
       </c>
-      <c r="I40" s="22"/>
-      <c r="J40" s="22"/>
-      <c r="K40" s="22"/>
-      <c r="L40" s="22"/>
-      <c r="M40" s="22"/>
-    </row>
-    <row r="41" spans="1:13">
-      <c r="I41" s="22"/>
-      <c r="J41" s="22"/>
-      <c r="K41" s="22"/>
-      <c r="L41" s="22"/>
-      <c r="M41" s="22"/>
+      <c r="C41" t="s">
+        <v>108</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="18">
-    <mergeCell ref="O19:O20"/>
-    <mergeCell ref="P19:P20"/>
-    <mergeCell ref="I38:I39"/>
-    <mergeCell ref="A36:B36"/>
-    <mergeCell ref="A35:B35"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="A24:B24"/>
+  <mergeCells count="17">
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="A17:B17"/>
     <mergeCell ref="A18:B18"/>
     <mergeCell ref="A16:B16"/>
+    <mergeCell ref="O19:O20"/>
+    <mergeCell ref="P19:P20"/>
+    <mergeCell ref="I37:I38"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="A24:B24"/>
     <mergeCell ref="A19:B19"/>
     <mergeCell ref="A20:B20"/>
     <mergeCell ref="A21:B21"/>
@@ -1280,482 +1442,483 @@
   <dimension ref="F1:J28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col min="9" max="9" width="30.1640625" customWidth="1"/>
+    <col min="6" max="6" width="36.5" customWidth="1"/>
+    <col min="9" max="9" width="61.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="6:10">
-      <c r="F1" s="20" t="s">
+      <c r="F1" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="G1" s="20" t="s">
+      <c r="G1" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="H1" s="20" t="s">
+      <c r="H1" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="I1" s="20" t="s">
+      <c r="I1" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="J1" s="20" t="s">
+      <c r="J1" s="15" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="2" spans="6:10">
-      <c r="F2" s="21" t="s">
+      <c r="F2" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="G2" s="21" t="s">
+      <c r="G2" s="16" t="s">
         <v>81</v>
       </c>
-      <c r="H2" s="21" t="s">
+      <c r="H2" s="16" t="s">
         <v>81</v>
       </c>
-      <c r="I2" s="21" t="s">
+      <c r="I2" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="J2" s="21" t="s">
+      <c r="J2" s="16" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="3" spans="6:10">
-      <c r="F3" s="18" t="s">
+      <c r="F3" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="G3" s="19">
+      <c r="G3" s="14">
         <v>1457</v>
       </c>
-      <c r="H3" s="19">
+      <c r="H3" s="14">
         <v>3201</v>
       </c>
-      <c r="I3" s="19" t="s">
+      <c r="I3" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="J3" s="19" t="s">
+      <c r="J3" s="14" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="4" spans="6:10">
-      <c r="F4" s="18" t="s">
+      <c r="F4" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="G4" s="19">
+      <c r="G4" s="14">
         <v>2909</v>
       </c>
-      <c r="H4" s="19">
+      <c r="H4" s="14">
         <v>2320</v>
       </c>
-      <c r="I4" s="19" t="s">
+      <c r="I4" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="J4" s="19" t="s">
+      <c r="J4" s="14" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="5" spans="6:10">
-      <c r="F5" s="18" t="s">
+      <c r="F5" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="G5" s="19">
+      <c r="G5" s="14">
         <v>1400</v>
       </c>
-      <c r="H5" s="19">
+      <c r="H5" s="14">
         <v>3024</v>
       </c>
-      <c r="I5" s="19" t="s">
+      <c r="I5" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="J5" s="19" t="s">
+      <c r="J5" s="14" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="6" spans="6:10">
-      <c r="F6" s="18" t="s">
+      <c r="F6" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="G6" s="19">
+      <c r="G6" s="14">
         <v>4067</v>
       </c>
-      <c r="H6" s="19">
+      <c r="H6" s="14">
         <v>1876</v>
       </c>
-      <c r="I6" s="19" t="s">
+      <c r="I6" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="J6" s="19" t="s">
+      <c r="J6" s="14" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="7" spans="6:10">
-      <c r="F7" s="18" t="s">
+      <c r="F7" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="G7" s="19">
+      <c r="G7" s="14">
         <v>1226</v>
       </c>
-      <c r="H7" s="19">
+      <c r="H7" s="14">
         <v>3005</v>
       </c>
-      <c r="I7" s="19" t="s">
+      <c r="I7" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="J7" s="19" t="s">
+      <c r="J7" s="14" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="8" spans="6:10">
-      <c r="F8" s="18" t="s">
+      <c r="F8" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="G8" s="19">
+      <c r="G8" s="14">
         <v>1232</v>
       </c>
-      <c r="H8" s="19">
+      <c r="H8" s="14">
         <v>2444</v>
       </c>
-      <c r="I8" s="19" t="s">
+      <c r="I8" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="J8" s="19" t="s">
+      <c r="J8" s="14" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="9" spans="6:10">
-      <c r="F9" s="18" t="s">
+      <c r="F9" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="G9" s="19">
+      <c r="G9" s="14">
         <v>737</v>
       </c>
-      <c r="H9" s="19">
+      <c r="H9" s="14">
         <v>3817</v>
       </c>
-      <c r="I9" s="19" t="s">
+      <c r="I9" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="J9" s="19" t="s">
+      <c r="J9" s="14" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="10" spans="6:10">
-      <c r="F10" s="18" t="s">
+      <c r="F10" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="G10" s="19">
+      <c r="G10" s="14">
         <v>692</v>
       </c>
-      <c r="H10" s="19">
+      <c r="H10" s="14">
         <v>2362</v>
       </c>
-      <c r="I10" s="19" t="s">
+      <c r="I10" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="J10" s="19" t="s">
+      <c r="J10" s="14" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="11" spans="6:10">
-      <c r="F11" s="18" t="s">
+      <c r="F11" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="G11" s="19">
+      <c r="G11" s="14">
         <v>1290</v>
       </c>
-      <c r="H11" s="19">
+      <c r="H11" s="14">
         <v>4017</v>
       </c>
-      <c r="I11" s="19" t="s">
+      <c r="I11" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="J11" s="19" t="s">
+      <c r="J11" s="14" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="12" spans="6:10">
-      <c r="F12" s="18" t="s">
+      <c r="F12" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="G12" s="19">
+      <c r="G12" s="14">
         <v>795</v>
       </c>
-      <c r="H12" s="19">
+      <c r="H12" s="14">
         <v>2103</v>
       </c>
-      <c r="I12" s="19" t="s">
+      <c r="I12" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="J12" s="19" t="s">
+      <c r="J12" s="14" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="13" spans="6:10">
-      <c r="F13" s="18" t="s">
+      <c r="F13" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="G13" s="19">
+      <c r="G13" s="14">
         <v>2444</v>
       </c>
-      <c r="H13" s="19">
+      <c r="H13" s="14">
         <v>5540</v>
       </c>
-      <c r="I13" s="19" t="s">
+      <c r="I13" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="J13" s="19" t="s">
+      <c r="J13" s="14" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="14" spans="6:10">
-      <c r="F14" s="18" t="s">
+      <c r="F14" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="G14" s="19">
+      <c r="G14" s="14">
         <v>1174</v>
       </c>
-      <c r="H14" s="19">
+      <c r="H14" s="14">
         <v>2261</v>
       </c>
-      <c r="I14" s="19" t="s">
+      <c r="I14" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="J14" s="19" t="s">
+      <c r="J14" s="14" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="15" spans="6:10">
-      <c r="F15" s="18" t="s">
+      <c r="F15" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="G15" s="19">
+      <c r="G15" s="14">
         <v>8989</v>
       </c>
-      <c r="H15" s="19">
+      <c r="H15" s="14">
         <v>7455</v>
       </c>
-      <c r="I15" s="19" t="s">
+      <c r="I15" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="J15" s="19" t="s">
+      <c r="J15" s="14" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="16" spans="6:10">
-      <c r="F16" s="18" t="s">
+      <c r="F16" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="G16" s="19">
+      <c r="G16" s="14">
         <v>2741</v>
       </c>
-      <c r="H16" s="19">
+      <c r="H16" s="14">
         <v>9785</v>
       </c>
-      <c r="I16" s="19" t="s">
+      <c r="I16" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="J16" s="19" t="s">
+      <c r="J16" s="14" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="17" spans="6:10">
-      <c r="F17" s="18" t="s">
+      <c r="F17" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="G17" s="19">
+      <c r="G17" s="14">
         <v>3675</v>
       </c>
-      <c r="H17" s="19">
+      <c r="H17" s="14">
         <v>4367</v>
       </c>
-      <c r="I17" s="19" t="s">
+      <c r="I17" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="J17" s="19" t="s">
+      <c r="J17" s="14" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="18" spans="6:10">
-      <c r="F18" s="18" t="s">
+      <c r="F18" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="G18" s="19">
+      <c r="G18" s="14">
         <v>1443</v>
       </c>
-      <c r="H18" s="19">
+      <c r="H18" s="14">
         <v>4511</v>
       </c>
-      <c r="I18" s="19" t="s">
+      <c r="I18" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="J18" s="19" t="s">
+      <c r="J18" s="14" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="19" spans="6:10">
-      <c r="F19" s="18" t="s">
+      <c r="F19" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="G19" s="19">
+      <c r="G19" s="14">
         <v>1031</v>
       </c>
-      <c r="H19" s="19">
+      <c r="H19" s="14">
         <v>2285</v>
       </c>
-      <c r="I19" s="19" t="s">
+      <c r="I19" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="J19" s="19" t="s">
+      <c r="J19" s="14" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="20" spans="6:10">
-      <c r="F20" s="18" t="s">
+      <c r="F20" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="G20" s="19">
+      <c r="G20" s="14">
         <v>915</v>
       </c>
-      <c r="H20" s="19">
+      <c r="H20" s="14">
         <v>2829</v>
       </c>
-      <c r="I20" s="19" t="s">
+      <c r="I20" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="J20" s="19" t="s">
+      <c r="J20" s="14" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="21" spans="6:10">
-      <c r="F21" s="18" t="s">
+      <c r="F21" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="G21" s="19">
+      <c r="G21" s="14">
         <v>7073</v>
       </c>
-      <c r="H21" s="19">
+      <c r="H21" s="14">
         <v>1049</v>
       </c>
-      <c r="I21" s="19" t="s">
+      <c r="I21" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="J21" s="19" t="s">
+      <c r="J21" s="14" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="22" spans="6:10">
-      <c r="F22" s="18" t="s">
+      <c r="F22" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="G22" s="19">
+      <c r="G22" s="14">
         <v>578</v>
       </c>
-      <c r="H22" s="19">
+      <c r="H22" s="14">
         <v>3002</v>
       </c>
-      <c r="I22" s="19" t="s">
+      <c r="I22" s="14" t="s">
         <v>64</v>
       </c>
-      <c r="J22" s="19" t="s">
+      <c r="J22" s="14" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="23" spans="6:10">
-      <c r="F23" s="18" t="s">
+      <c r="F23" s="13" t="s">
         <v>65</v>
       </c>
-      <c r="G23" s="19">
+      <c r="G23" s="14">
         <v>4589</v>
       </c>
-      <c r="H23" s="19">
+      <c r="H23" s="14">
         <v>2729</v>
       </c>
-      <c r="I23" s="19" t="s">
+      <c r="I23" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="J23" s="19" t="s">
+      <c r="J23" s="14" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="24" spans="6:10">
-      <c r="F24" s="18" t="s">
+      <c r="F24" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="G24" s="19">
+      <c r="G24" s="14">
         <v>1264</v>
       </c>
-      <c r="H24" s="19">
+      <c r="H24" s="14">
         <v>2243</v>
       </c>
-      <c r="I24" s="19" t="s">
+      <c r="I24" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="J24" s="19" t="s">
+      <c r="J24" s="14" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="25" spans="6:10">
-      <c r="F25" s="18" t="s">
+      <c r="F25" s="13" t="s">
         <v>69</v>
       </c>
-      <c r="G25" s="19">
+      <c r="G25" s="14">
         <v>1590</v>
       </c>
-      <c r="H25" s="19">
+      <c r="H25" s="14">
         <v>3670</v>
       </c>
-      <c r="I25" s="19" t="s">
+      <c r="I25" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="J25" s="19" t="s">
+      <c r="J25" s="14" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="26" spans="6:10">
-      <c r="F26" s="18" t="s">
+      <c r="F26" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="G26" s="19">
+      <c r="G26" s="14">
         <v>12129</v>
       </c>
-      <c r="H26" s="19">
+      <c r="H26" s="14">
         <v>2726</v>
       </c>
-      <c r="I26" s="19" t="s">
+      <c r="I26" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="J26" s="19" t="s">
+      <c r="J26" s="14" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="27" spans="6:10">
-      <c r="F27" s="18" t="s">
+      <c r="F27" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="G27" s="19">
+      <c r="G27" s="14">
         <v>1180</v>
       </c>
-      <c r="H27" s="19">
+      <c r="H27" s="14">
         <v>2285</v>
       </c>
-      <c r="I27" s="19" t="s">
+      <c r="I27" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="J27" s="19" t="s">
+      <c r="J27" s="14" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="28" spans="6:10">
-      <c r="F28" s="18" t="s">
+      <c r="F28" s="13" t="s">
         <v>75</v>
       </c>
-      <c r="G28" s="19">
+      <c r="G28" s="14">
         <v>1825</v>
       </c>
-      <c r="H28" s="19">
+      <c r="H28" s="14">
         <v>5093</v>
       </c>
-      <c r="I28" s="19" t="s">
+      <c r="I28" s="14" t="s">
         <v>76</v>
       </c>
-      <c r="J28" s="19" t="s">
+      <c r="J28" s="14" t="s">
         <v>54</v>
       </c>
     </row>
@@ -1769,129 +1932,129 @@
   <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" customWidth="1"/>
     <col min="3" max="3" width="9.5" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="15" t="s">
         <v>77</v>
       </c>
-      <c r="B1" s="20" t="s">
+      <c r="B1" s="15" t="s">
         <v>79</v>
       </c>
-      <c r="C1" s="20" t="s">
+      <c r="C1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="20" t="s">
+      <c r="D1" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="20" t="s">
+      <c r="E1" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="F1" s="20" t="s">
+      <c r="F1" s="15" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="16" t="s">
         <v>78</v>
       </c>
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="16" t="s">
         <v>78</v>
       </c>
-      <c r="C2" s="21" t="s">
+      <c r="C2" s="16" t="s">
         <v>86</v>
       </c>
-      <c r="D2" s="21" t="s">
+      <c r="D2" s="16" t="s">
         <v>86</v>
       </c>
-      <c r="E2" s="21" t="s">
+      <c r="E2" s="16" t="s">
         <v>81</v>
       </c>
-      <c r="F2" s="21" t="s">
+      <c r="F2" s="16" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="17" t="s">
         <v>82</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="17" t="s">
         <v>83</v>
       </c>
-      <c r="C3" s="22">
+      <c r="C3" s="17">
         <v>2225.2139999999999</v>
       </c>
-      <c r="D3" s="22">
+      <c r="D3" s="17">
         <v>2179.788</v>
       </c>
-      <c r="E3" s="22">
+      <c r="E3" s="17">
         <v>14</v>
       </c>
-      <c r="F3" s="22">
+      <c r="F3" s="17">
         <v>582.5729</v>
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="17" t="s">
         <v>82</v>
       </c>
-      <c r="B4" s="22" t="s">
+      <c r="B4" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="C4" s="22">
+      <c r="C4" s="17">
         <v>3107.6669999999999</v>
       </c>
-      <c r="D4" s="22">
+      <c r="D4" s="17">
         <v>3424.2289999999998</v>
       </c>
-      <c r="E4" s="22">
+      <c r="E4" s="17">
         <v>12</v>
       </c>
-      <c r="F4" s="22">
+      <c r="F4" s="17">
         <v>988.4896</v>
       </c>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="17" t="s">
         <v>85</v>
       </c>
-      <c r="B5" s="22" t="s">
+      <c r="B5" s="17" t="s">
         <v>83</v>
       </c>
-      <c r="C5" s="22">
+      <c r="C5" s="17">
         <v>3800.7139999999999</v>
       </c>
-      <c r="D5" s="22">
+      <c r="D5" s="17">
         <v>2302.078</v>
       </c>
-      <c r="E5" s="22">
+      <c r="E5" s="17">
         <v>14</v>
       </c>
-      <c r="F5" s="22">
+      <c r="F5" s="17">
         <v>615.25620000000004</v>
       </c>
     </row>
     <row r="6" spans="1:6">
-      <c r="A6" s="22" t="s">
+      <c r="A6" s="17" t="s">
         <v>85</v>
       </c>
-      <c r="B6" s="22" t="s">
+      <c r="B6" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="C6" s="22">
+      <c r="C6" s="17">
         <v>3065.75</v>
       </c>
-      <c r="D6" s="22">
+      <c r="D6" s="17">
         <v>1148.4829999999999</v>
       </c>
-      <c r="E6" s="22">
+      <c r="E6" s="17">
         <v>12</v>
       </c>
-      <c r="F6" s="22">
+      <c r="F6" s="17">
         <v>331.5385</v>
       </c>
     </row>
@@ -1918,70 +2081,70 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="15" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="20" t="s">
+      <c r="B1" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="20" t="s">
+      <c r="C1" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="D1" s="20" t="s">
+      <c r="D1" s="15" t="s">
         <v>91</v>
       </c>
-      <c r="E1" s="20" t="s">
+      <c r="E1" s="15" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:10">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="16" t="s">
         <v>86</v>
       </c>
-      <c r="C2" s="21" t="s">
+      <c r="C2" s="16" t="s">
         <v>86</v>
       </c>
-      <c r="D2" s="21" t="s">
+      <c r="D2" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="E2" s="21" t="s">
+      <c r="E2" s="16" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="3" spans="1:10">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="17" t="s">
         <v>93</v>
       </c>
-      <c r="B3" s="22">
+      <c r="B3" s="17">
         <v>94</v>
       </c>
-      <c r="C3" s="22">
+      <c r="C3" s="17">
         <v>0.6250464</v>
       </c>
-      <c r="D3" s="22" t="s">
+      <c r="D3" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="E3" s="22" t="s">
+      <c r="E3" s="17" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="4" spans="1:10">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="17" t="s">
         <v>96</v>
       </c>
-      <c r="B4" s="22">
+      <c r="B4" s="17">
         <v>74</v>
       </c>
-      <c r="C4" s="22">
+      <c r="C4" s="17">
         <v>0.62510560000000004</v>
       </c>
-      <c r="D4" s="22" t="s">
+      <c r="D4" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="E4" s="22" t="s">
+      <c r="E4" s="17" t="s">
         <v>95</v>
       </c>
     </row>
@@ -2163,17 +2326,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="17c61571-0fe9-4ceb-9b66-2de528a072b1" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="12423bc7-10a6-4cd4-bb27-11b0289f8e4d">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008D551129DB99E8438FE6EF309F08C354" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="7dc744bdf5b6a0bc20f5fdcb351cc095">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="12423bc7-10a6-4cd4-bb27-11b0289f8e4d" xmlns:ns3="17c61571-0fe9-4ceb-9b66-2de528a072b1" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3890b32a57b45779b4d4b2e999852729" ns2:_="" ns3:_="">
     <xsd:import namespace="12423bc7-10a6-4cd4-bb27-11b0289f8e4d"/>
@@ -2386,6 +2538,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="17c61571-0fe9-4ceb-9b66-2de528a072b1" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="12423bc7-10a6-4cd4-bb27-11b0289f8e4d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -2396,23 +2559,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{29883378-2D7B-4326-849D-497DD2210F57}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="17c61571-0fe9-4ceb-9b66-2de528a072b1"/>
-    <ds:schemaRef ds:uri="12423bc7-10a6-4cd4-bb27-11b0289f8e4d"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E34AA185-27E2-43D0-9F42-CE10CD9A7418}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2431,6 +2577,23 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{29883378-2D7B-4326-849D-497DD2210F57}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="17c61571-0fe9-4ceb-9b66-2de528a072b1"/>
+    <ds:schemaRef ds:uri="12423bc7-10a6-4cd4-bb27-11b0289f8e4d"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{349E94C1-8144-465E-BEF6-F5255DE36DE4}">
   <ds:schemaRefs>

</xml_diff>